<commit_message>
Elde tutma optimizasyonu + km etkisi analizi
- a×h matrisi: alım yaşı × tutma süresi yıllık bileşik kayıp (Türkiye ort.)
- Bulgu: keskin satış eşiği yok, uzun tutmak giriş maliyetini amortize eder
- Km etkisi log-konkav: +20k km, 20k km'li araçta %7.2, 150k'lıda %1.3
- Kombine senaryolar: 10/20/30k km-yıl kullanım profilleri
- 6 tutarlılık testi (teleskop, ampirik beta doğrulaması dahil)
</commit_message>
<xml_diff>
--- a/reports/rapor_tum_araclar.xlsx
+++ b/reports/rapor_tum_araclar.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modeller" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Turkiye Ortalamasi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="USD-TUFE Kohort" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guncel Sifir Fiyatlar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motor Varyantlari" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodoloji" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapsam Disi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elde Tutma &amp; Km" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="USD-TUFE Kohort" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guncel Sifir Fiyatlar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motor Varyantlari" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodoloji" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapsam Disi" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,8 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -124,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,6 +143,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8352,6 +8360,372 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ELDE TUTMA OPTIMIZASYONU — 'a yasinda al, h yil kullan' yillik deger kaybi % (Turkiye ort., yas-tipik km)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Okuma: hucre degeri = yillik bilesik kayip. Sag/asagi gittikce dusuyor -&gt; uzun tutmak giris maliyetini amortize eder, keskin bir 'optimal satis yili' yoktur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Alim Yasi \ Tutma (yil)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="H5" s="15" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="I5" s="15" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="I6" s="15" t="n">
+        <v>7.13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>7.26</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>6.87</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="I8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>KM ETKISI — ayni +20.000 km'nin maliyeti mevcut km'ye gore (log-konkav: ilk km'ler daha pahali)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Mevcut km</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>+20.000 km'nin maliyeti (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>150000</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>200000</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>KOMBINE SENARYO (4 yil tutma): 10k km/yil surerken yillik kayip %6.2-6.6; 20k km/yil: %6.9-7.7; 30k km/yil: %7.5-8.6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Verideki tipik kullanim: ~18.000 km/yil. Km betasi (medyan): -0.109 (log-log).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>CIKARIMLAR: (1) Uzun tutmak her zaman marjinal olarak daha ucuz — 'su yilda sat' esigi yok, kazanc yilda ~0.1-0.3 puanla azalarak surer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>(2) Cok km yapacaksan yasli/yuksek km arac al: ayni 20.000 km, 20k km'li araca %7.2, 150k km'li araca %1.3'e mal oluyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>(3) Az km yapiyorsan genc arac almak affedilir; cok km yapiyorsan genc arac cift ceza (yas + pahali km'ler).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -11505,7 +11879,7 @@
         <v>-0.3</v>
       </c>
       <c r="L72" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>48</v>
@@ -13704,7 +14078,7 @@
         <v>-0.1</v>
       </c>
       <c r="J121" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K121" s="3" t="n">
         <v>19.8</v>
@@ -14643,7 +15017,7 @@
         <v>44354</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I142" s="3" t="n">
         <v>10.6</v>
@@ -16376,7 +16750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19917,7 +20291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25291,7 +25665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25395,7 +25769,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>